<commit_message>
UK daily ratings for 2026-06-02
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-06-02.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-06-02.xlsx
@@ -773,7 +773,7 @@
         <v>4</v>
       </c>
       <c r="J6" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="K6" t="n">
         <v>47</v>
@@ -785,7 +785,7 @@
         <v>135.52</v>
       </c>
       <c r="N6" t="n">
-        <v>36.3</v>
+        <v>35.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
         <v>8</v>
       </c>
       <c r="J7" t="n">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="K7" t="n">
         <v>45</v>
@@ -845,7 +845,7 @@
         <v>135.52</v>
       </c>
       <c r="N7" t="n">
-        <v>35.7</v>
+        <v>34.2</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="K8" t="n">
         <v>48</v>
@@ -905,7 +905,7 @@
         <v>135.52</v>
       </c>
       <c r="N8" t="n">
-        <v>33</v>
+        <v>29.4</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1313,7 +1313,7 @@
         <v>6</v>
       </c>
       <c r="J15" t="n">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="K15" t="n">
         <v>60</v>
@@ -1323,7 +1323,7 @@
         <v>162.53</v>
       </c>
       <c r="N15" t="n">
-        <v>71</v>
+        <v>66.3</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="16">
@@ -1371,7 +1371,7 @@
         <v>4</v>
       </c>
       <c r="J16" t="n">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="K16" t="n">
         <v>58</v>
@@ -1383,7 +1383,7 @@
         <v>162.53</v>
       </c>
       <c r="N16" t="n">
-        <v>68</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>-0.5</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="17">
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1611,7 +1611,7 @@
         <v>6</v>
       </c>
       <c r="J20" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="K20" t="n">
         <v>60</v>
@@ -1623,7 +1623,7 @@
         <v>162.53</v>
       </c>
       <c r="N20" t="n">
-        <v>63.8</v>
+        <v>61.3</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1791,7 +1791,7 @@
         <v>5</v>
       </c>
       <c r="J23" t="n">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="K23" t="n">
         <v>46</v>
@@ -1803,7 +1803,7 @@
         <v>162.53</v>
       </c>
       <c r="N23" t="n">
-        <v>42.4</v>
+        <v>38.9</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="24">
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1911,7 +1911,7 @@
         <v>4</v>
       </c>
       <c r="J25" t="n">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K25" t="n">
         <v>56</v>
@@ -1923,7 +1923,7 @@
         <v>162.53</v>
       </c>
       <c r="N25" t="n">
-        <v>24.8</v>
+        <v>22.5</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2209,7 +2209,7 @@
         <v>3</v>
       </c>
       <c r="J30" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="K30" t="n">
         <v>62</v>
@@ -2221,7 +2221,7 @@
         <v>61.47</v>
       </c>
       <c r="N30" t="n">
-        <v>18.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -2269,7 +2269,7 @@
         <v>3</v>
       </c>
       <c r="J31" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="K31" t="n">
         <v>54</v>
@@ -2281,7 +2281,7 @@
         <v>61.47</v>
       </c>
       <c r="N31" t="n">
-        <v>-8.699999999999999</v>
+        <v>-13.3</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -2318,34 +2318,36 @@
         <v>6</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Hyrcanian (IRE)</t>
+          <t>Auntie Jo</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J32" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K32" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
         <v>60.84</v>
       </c>
-      <c r="N32" t="inlineStr"/>
+      <c r="N32" t="n">
+        <v>49.7</v>
+      </c>
       <c r="O32" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>-9.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -2374,34 +2376,38 @@
         <v>6</v>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Lets Go Hugo (IRE)</t>
+          <t>A Lady Forever</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J33" t="n">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="K33" t="n">
-        <v>53</v>
-      </c>
-      <c r="L33" t="inlineStr"/>
+        <v>45</v>
+      </c>
+      <c r="L33" t="n">
+        <v>2.75</v>
+      </c>
       <c r="M33" t="n">
         <v>60.84</v>
       </c>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" t="n">
+        <v>41.9</v>
+      </c>
       <c r="O33" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>-9.5</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="34">
@@ -2430,28 +2436,30 @@
         <v>6</v>
       </c>
       <c r="G34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Auntie Jo</t>
+          <t>What What What</t>
         </is>
       </c>
       <c r="I34" t="n">
         <v>4</v>
       </c>
       <c r="J34" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K34" t="n">
-        <v>50</v>
-      </c>
-      <c r="L34" t="inlineStr"/>
+        <v>51</v>
+      </c>
+      <c r="L34" t="n">
+        <v>3.75</v>
+      </c>
       <c r="M34" t="n">
         <v>60.84</v>
       </c>
       <c r="N34" t="n">
-        <v>56.9</v>
+        <v>42.1</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -2459,7 +2467,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -2488,30 +2496,30 @@
         <v>6</v>
       </c>
       <c r="G35" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>A Lady Forever</t>
+          <t>Jeany May</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J35" t="n">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="K35" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="L35" t="n">
-        <v>2.75</v>
+        <v>3.9</v>
       </c>
       <c r="M35" t="n">
         <v>60.84</v>
       </c>
       <c r="N35" t="n">
-        <v>41.9</v>
+        <v>39.5</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -2519,7 +2527,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -2548,30 +2556,30 @@
         <v>6</v>
       </c>
       <c r="G36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>What What What</t>
+          <t>Barneys Bay</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J36" t="n">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="K36" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="L36" t="n">
-        <v>3.75</v>
+        <v>4.4</v>
       </c>
       <c r="M36" t="n">
         <v>60.84</v>
       </c>
       <c r="N36" t="n">
-        <v>42.1</v>
+        <v>33.5</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -2579,7 +2587,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -2608,30 +2616,30 @@
         <v>6</v>
       </c>
       <c r="G37" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Jeany May</t>
+          <t>Desert Champion (IRE)</t>
         </is>
       </c>
       <c r="I37" t="n">
         <v>4</v>
       </c>
       <c r="J37" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K37" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="L37" t="n">
-        <v>3.9</v>
+        <v>7.4</v>
       </c>
       <c r="M37" t="n">
         <v>60.84</v>
       </c>
       <c r="N37" t="n">
-        <v>39.5</v>
+        <v>26.4</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -2668,30 +2676,30 @@
         <v>6</v>
       </c>
       <c r="G38" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Barneys Bay</t>
+          <t>Bishops Glory (IRE)</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J38" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K38" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="L38" t="n">
-        <v>4.4</v>
+        <v>9.65</v>
       </c>
       <c r="M38" t="n">
         <v>60.84</v>
       </c>
       <c r="N38" t="n">
-        <v>33.5</v>
+        <v>14.5</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -2728,30 +2736,30 @@
         <v>6</v>
       </c>
       <c r="G39" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Desert Champion (IRE)</t>
+          <t>Posh Maisie (IRE)</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J39" t="n">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="K39" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="L39" t="n">
-        <v>7.4</v>
+        <v>10.15</v>
       </c>
       <c r="M39" t="n">
         <v>60.84</v>
       </c>
       <c r="N39" t="n">
-        <v>26.4</v>
+        <v>9.4</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -2787,40 +2795,24 @@
       <c r="F40" t="n">
         <v>6</v>
       </c>
-      <c r="G40" t="n">
-        <v>7</v>
-      </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Bishops Glory (IRE)</t>
-        </is>
-      </c>
-      <c r="I40" t="n">
-        <v>6</v>
-      </c>
-      <c r="J40" t="n">
-        <v>129</v>
-      </c>
-      <c r="K40" t="n">
-        <v>47</v>
-      </c>
-      <c r="L40" t="n">
-        <v>9.65</v>
-      </c>
-      <c r="M40" t="n">
-        <v>60.84</v>
-      </c>
-      <c r="N40" t="n">
-        <v>14.5</v>
-      </c>
+          <t>Lets Go Hugo (IRE)</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P40" t="n">
-        <v>0</v>
-      </c>
+      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2847,40 +2839,24 @@
       <c r="F41" t="n">
         <v>6</v>
       </c>
-      <c r="G41" t="n">
-        <v>8</v>
-      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Posh Maisie (IRE)</t>
-        </is>
-      </c>
-      <c r="I41" t="n">
-        <v>5</v>
-      </c>
-      <c r="J41" t="n">
-        <v>127</v>
-      </c>
-      <c r="K41" t="n">
-        <v>45</v>
-      </c>
-      <c r="L41" t="n">
-        <v>10.15</v>
-      </c>
-      <c r="M41" t="n">
-        <v>60.84</v>
-      </c>
-      <c r="N41" t="n">
-        <v>9.4</v>
-      </c>
+          <t>Hyrcanian (IRE)</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P41" t="n">
-        <v>0</v>
-      </c>
+      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2977,7 +2953,7 @@
         <v>6</v>
       </c>
       <c r="J43" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="K43" t="n">
         <v>60</v>
@@ -2989,7 +2965,7 @@
         <v>101.42</v>
       </c>
       <c r="N43" t="n">
-        <v>50.1</v>
+        <v>45.3</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -2997,7 +2973,7 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="44">
@@ -3057,7 +3033,7 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -3097,7 +3073,7 @@
         <v>5</v>
       </c>
       <c r="J45" t="n">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="K45" t="n">
         <v>74</v>
@@ -3109,7 +3085,7 @@
         <v>101.42</v>
       </c>
       <c r="N45" t="n">
-        <v>54.1</v>
+        <v>49.7</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -3117,7 +3093,7 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -3157,7 +3133,7 @@
         <v>5</v>
       </c>
       <c r="J46" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="K46" t="n">
         <v>63</v>
@@ -3169,7 +3145,7 @@
         <v>101.42</v>
       </c>
       <c r="N46" t="n">
-        <v>43.5</v>
+        <v>40</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -3177,7 +3153,7 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="47">
@@ -3237,7 +3213,7 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
@@ -3297,7 +3273,7 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -3337,19 +3313,19 @@
         <v>6</v>
       </c>
       <c r="J49" t="n">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="K49" t="n">
         <v>74</v>
       </c>
       <c r="L49" t="n">
-        <v>6.8</v>
+        <v>6.800000000000001</v>
       </c>
       <c r="M49" t="n">
         <v>101.42</v>
       </c>
       <c r="N49" t="n">
-        <v>46.7</v>
+        <v>45</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -3417,7 +3393,7 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -3463,7 +3439,7 @@
         <v>72</v>
       </c>
       <c r="L51" t="n">
-        <v>8.699999999999999</v>
+        <v>8.700000000000001</v>
       </c>
       <c r="M51" t="n">
         <v>101.42</v>
@@ -3477,7 +3453,7 @@
         </is>
       </c>
       <c r="P51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -3577,7 +3553,7 @@
         <v>8</v>
       </c>
       <c r="J53" t="n">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="K53" t="n">
         <v>64</v>
@@ -3589,7 +3565,7 @@
         <v>101.42</v>
       </c>
       <c r="N53" t="n">
-        <v>27.3</v>
+        <v>24</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -3626,34 +3602,36 @@
         <v>6</v>
       </c>
       <c r="G54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Bantz (IRE)</t>
+          <t>Dinah Myte</t>
         </is>
       </c>
       <c r="I54" t="n">
         <v>4</v>
       </c>
       <c r="J54" t="n">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="K54" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="n">
         <v>102.54</v>
       </c>
-      <c r="N54" t="inlineStr"/>
+      <c r="N54" t="n">
+        <v>45.5</v>
+      </c>
       <c r="O54" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P54" t="n">
-        <v>-14</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="55">
@@ -3682,28 +3660,30 @@
         <v>6</v>
       </c>
       <c r="G55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Dinah Myte</t>
+          <t>Barleybrown</t>
         </is>
       </c>
       <c r="I55" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J55" t="n">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="K55" t="n">
-        <v>46</v>
-      </c>
-      <c r="L55" t="inlineStr"/>
+        <v>53</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.5</v>
+      </c>
       <c r="M55" t="n">
         <v>102.54</v>
       </c>
       <c r="N55" t="n">
-        <v>45.5</v>
+        <v>52.8</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
@@ -3711,7 +3691,7 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>-6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -3740,30 +3720,30 @@
         <v>6</v>
       </c>
       <c r="G56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Barleybrown</t>
+          <t>Abu Royal (IRE)</t>
         </is>
       </c>
       <c r="I56" t="n">
         <v>6</v>
       </c>
       <c r="J56" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="K56" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="L56" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="M56" t="n">
         <v>102.54</v>
       </c>
       <c r="N56" t="n">
-        <v>52.8</v>
+        <v>44.9</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -3771,7 +3751,7 @@
         </is>
       </c>
       <c r="P56" t="n">
-        <v>1</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="57">
@@ -3800,30 +3780,30 @@
         <v>6</v>
       </c>
       <c r="G57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Abu Royal (IRE)</t>
+          <t>Volenti (IRE)</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J57" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="K57" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="L57" t="n">
-        <v>0.6</v>
+        <v>1.6</v>
       </c>
       <c r="M57" t="n">
         <v>102.54</v>
       </c>
       <c r="N57" t="n">
-        <v>44.9</v>
+        <v>45.8</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -3831,7 +3811,7 @@
         </is>
       </c>
       <c r="P57" t="n">
-        <v>-5</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="58">
@@ -3860,15 +3840,15 @@
         <v>6</v>
       </c>
       <c r="G58" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Volenti (IRE)</t>
+          <t>Little Ted</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J58" t="n">
         <v>130</v>
@@ -3877,13 +3857,13 @@
         <v>50</v>
       </c>
       <c r="L58" t="n">
-        <v>1.6</v>
+        <v>1.75</v>
       </c>
       <c r="M58" t="n">
         <v>102.54</v>
       </c>
       <c r="N58" t="n">
-        <v>45.8</v>
+        <v>45.7</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -3920,30 +3900,30 @@
         <v>6</v>
       </c>
       <c r="G59" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Little Ted</t>
+          <t>Penny Mountain (IRE)</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J59" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K59" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="L59" t="n">
-        <v>1.75</v>
+        <v>1.85</v>
       </c>
       <c r="M59" t="n">
         <v>102.54</v>
       </c>
       <c r="N59" t="n">
-        <v>45.7</v>
+        <v>48.5</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -3951,7 +3931,7 @@
         </is>
       </c>
       <c r="P59" t="n">
-        <v>-1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="60">
@@ -3980,30 +3960,30 @@
         <v>6</v>
       </c>
       <c r="G60" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Penny Mountain (IRE)</t>
+          <t>Cable Beach</t>
         </is>
       </c>
       <c r="I60" t="n">
         <v>5</v>
       </c>
       <c r="J60" t="n">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="K60" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="L60" t="n">
-        <v>1.85</v>
+        <v>2</v>
       </c>
       <c r="M60" t="n">
         <v>102.54</v>
       </c>
       <c r="N60" t="n">
-        <v>50.4</v>
+        <v>42.9</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -4011,7 +3991,7 @@
         </is>
       </c>
       <c r="P60" t="n">
-        <v>4</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="61">
@@ -4040,30 +4020,30 @@
         <v>6</v>
       </c>
       <c r="G61" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Cable Beach</t>
+          <t>Mercurius Power (IRE)</t>
         </is>
       </c>
       <c r="I61" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J61" t="n">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="K61" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L61" t="n">
-        <v>2</v>
+        <v>2.15</v>
       </c>
       <c r="M61" t="n">
         <v>102.54</v>
       </c>
       <c r="N61" t="n">
-        <v>42.9</v>
+        <v>49.4</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -4071,7 +4051,7 @@
         </is>
       </c>
       <c r="P61" t="n">
-        <v>-3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62">
@@ -4100,30 +4080,30 @@
         <v>6</v>
       </c>
       <c r="G62" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Mercurius Power (IRE)</t>
+          <t>Wicklow Way (IRE)</t>
         </is>
       </c>
       <c r="I62" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J62" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K62" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L62" t="n">
-        <v>2.15</v>
+        <v>2.2</v>
       </c>
       <c r="M62" t="n">
         <v>102.54</v>
       </c>
       <c r="N62" t="n">
-        <v>49.4</v>
+        <v>48.1</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -4160,30 +4140,30 @@
         <v>6</v>
       </c>
       <c r="G63" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Wicklow Way (IRE)</t>
+          <t>First Encounter</t>
         </is>
       </c>
       <c r="I63" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J63" t="n">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="K63" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="L63" t="n">
-        <v>2.2</v>
+        <v>3.2</v>
       </c>
       <c r="M63" t="n">
         <v>102.54</v>
       </c>
       <c r="N63" t="n">
-        <v>48.1</v>
+        <v>36.1</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -4191,7 +4171,7 @@
         </is>
       </c>
       <c r="P63" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -4220,30 +4200,30 @@
         <v>6</v>
       </c>
       <c r="G64" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>First Encounter</t>
+          <t>Trais Fluors</t>
         </is>
       </c>
       <c r="I64" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="J64" t="n">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="K64" t="n">
         <v>51</v>
       </c>
       <c r="L64" t="n">
-        <v>3.2</v>
+        <v>4.199999999999999</v>
       </c>
       <c r="M64" t="n">
         <v>102.54</v>
       </c>
       <c r="N64" t="n">
-        <v>43.6</v>
+        <v>35.7</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -4251,7 +4231,7 @@
         </is>
       </c>
       <c r="P64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -4280,30 +4260,30 @@
         <v>6</v>
       </c>
       <c r="G65" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Trais Fluors</t>
+          <t>Rocket Rod (IRE)</t>
         </is>
       </c>
       <c r="I65" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J65" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="K65" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="L65" t="n">
-        <v>4.2</v>
+        <v>12.7</v>
       </c>
       <c r="M65" t="n">
         <v>102.54</v>
       </c>
       <c r="N65" t="n">
-        <v>41.3</v>
+        <v>23.1</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -4340,30 +4320,30 @@
         <v>6</v>
       </c>
       <c r="G66" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Rocket Rod (IRE)</t>
+          <t>Billyjoegold</t>
         </is>
       </c>
       <c r="I66" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J66" t="n">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="K66" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L66" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="M66" t="n">
         <v>102.54</v>
       </c>
       <c r="N66" t="n">
-        <v>23.1</v>
+        <v>14.9</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -4399,40 +4379,24 @@
       <c r="F67" t="n">
         <v>6</v>
       </c>
-      <c r="G67" t="n">
-        <v>13</v>
-      </c>
+      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Billyjoegold</t>
-        </is>
-      </c>
-      <c r="I67" t="n">
-        <v>4</v>
-      </c>
-      <c r="J67" t="n">
-        <v>127</v>
-      </c>
-      <c r="K67" t="n">
-        <v>47</v>
-      </c>
-      <c r="L67" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="M67" t="n">
-        <v>102.54</v>
-      </c>
-      <c r="N67" t="n">
-        <v>14.9</v>
-      </c>
+          <t>Bantz (IRE)</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P67" t="n">
-        <v>0</v>
-      </c>
+      <c r="P67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4649,7 +4613,7 @@
         <v>3</v>
       </c>
       <c r="J71" t="n">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="K71" t="n">
         <v>0</v>
@@ -4661,7 +4625,7 @@
         <v>132.72</v>
       </c>
       <c r="N71" t="n">
-        <v>24.7</v>
+        <v>24</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -4698,11 +4662,11 @@
         <v>4</v>
       </c>
       <c r="G72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Rosberg</t>
+          <t>Boleto (IRE)</t>
         </is>
       </c>
       <c r="I72" t="n">
@@ -4718,14 +4682,16 @@
       <c r="M72" t="n">
         <v>76.92</v>
       </c>
-      <c r="N72" t="inlineStr"/>
+      <c r="N72" t="n">
+        <v>60.2</v>
+      </c>
       <c r="O72" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P72" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -4754,11 +4720,11 @@
         <v>4</v>
       </c>
       <c r="G73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Boleto (IRE)</t>
+          <t>Shemiyla Star (IRE)</t>
         </is>
       </c>
       <c r="I73" t="n">
@@ -4770,12 +4736,14 @@
       <c r="K73" t="n">
         <v>0</v>
       </c>
-      <c r="L73" t="inlineStr"/>
+      <c r="L73" t="n">
+        <v>0.15</v>
+      </c>
       <c r="M73" t="n">
         <v>76.92</v>
       </c>
       <c r="N73" t="n">
-        <v>60.2</v>
+        <v>58.8</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
@@ -4812,30 +4780,30 @@
         <v>4</v>
       </c>
       <c r="G74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Shemiyla Star (IRE)</t>
+          <t>Kochella (IRE)</t>
         </is>
       </c>
       <c r="I74" t="n">
         <v>2</v>
       </c>
       <c r="J74" t="n">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="K74" t="n">
         <v>0</v>
       </c>
       <c r="L74" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="M74" t="n">
         <v>76.92</v>
       </c>
       <c r="N74" t="n">
-        <v>58.8</v>
+        <v>54.3</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -4872,30 +4840,30 @@
         <v>4</v>
       </c>
       <c r="G75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Kochella (IRE)</t>
+          <t>Avionics (IRE)</t>
         </is>
       </c>
       <c r="I75" t="n">
         <v>2</v>
       </c>
       <c r="J75" t="n">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="K75" t="n">
         <v>0</v>
       </c>
       <c r="L75" t="n">
-        <v>0.3</v>
+        <v>2.05</v>
       </c>
       <c r="M75" t="n">
         <v>76.92</v>
       </c>
       <c r="N75" t="n">
-        <v>54.3</v>
+        <v>53.4</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -4932,11 +4900,11 @@
         <v>4</v>
       </c>
       <c r="G76" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Avionics (IRE)</t>
+          <t>Inns And Out (IRE)</t>
         </is>
       </c>
       <c r="I76" t="n">
@@ -4949,13 +4917,13 @@
         <v>0</v>
       </c>
       <c r="L76" t="n">
-        <v>2.05</v>
+        <v>3.55</v>
       </c>
       <c r="M76" t="n">
         <v>76.92</v>
       </c>
       <c r="N76" t="n">
-        <v>53.4</v>
+        <v>47.5</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
@@ -4992,30 +4960,30 @@
         <v>4</v>
       </c>
       <c r="G77" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Inns And Out (IRE)</t>
+          <t>Desert Phantom</t>
         </is>
       </c>
       <c r="I77" t="n">
         <v>2</v>
       </c>
       <c r="J77" t="n">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="K77" t="n">
         <v>0</v>
       </c>
       <c r="L77" t="n">
-        <v>3.55</v>
+        <v>7.800000000000001</v>
       </c>
       <c r="M77" t="n">
         <v>76.92</v>
       </c>
       <c r="N77" t="n">
-        <v>47.5</v>
+        <v>30.3</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -5052,11 +5020,11 @@
         <v>4</v>
       </c>
       <c r="G78" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Desert Phantom</t>
+          <t>Raslan</t>
         </is>
       </c>
       <c r="I78" t="n">
@@ -5069,13 +5037,13 @@
         <v>0</v>
       </c>
       <c r="L78" t="n">
-        <v>7.8</v>
+        <v>11.55</v>
       </c>
       <c r="M78" t="n">
         <v>76.92</v>
       </c>
       <c r="N78" t="n">
-        <v>35.5</v>
+        <v>22.5</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
@@ -5111,40 +5079,24 @@
       <c r="F79" t="n">
         <v>4</v>
       </c>
-      <c r="G79" t="n">
-        <v>7</v>
-      </c>
+      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Raslan</t>
-        </is>
-      </c>
-      <c r="I79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J79" t="n">
-        <v>133</v>
-      </c>
-      <c r="K79" t="n">
-        <v>0</v>
-      </c>
-      <c r="L79" t="n">
-        <v>11.55</v>
-      </c>
-      <c r="M79" t="n">
-        <v>76.92</v>
-      </c>
-      <c r="N79" t="n">
-        <v>22.5</v>
-      </c>
+          <t>Rosberg</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P79" t="n">
-        <v>0</v>
-      </c>
+      <c r="P79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5172,34 +5124,36 @@
         <v>4</v>
       </c>
       <c r="G80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Irish Nectar</t>
+          <t>Rock Opera</t>
         </is>
       </c>
       <c r="I80" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J80" t="n">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="K80" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="n">
         <v>74.84</v>
       </c>
-      <c r="N80" t="inlineStr"/>
+      <c r="N80" t="n">
+        <v>78.90000000000001</v>
+      </c>
       <c r="O80" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P80" t="n">
-        <v>-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -5228,28 +5182,30 @@
         <v>4</v>
       </c>
       <c r="G81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Rock Opera</t>
+          <t>Alpha Capture (IRE)</t>
         </is>
       </c>
       <c r="I81" t="n">
         <v>6</v>
       </c>
       <c r="J81" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="K81" t="n">
-        <v>70</v>
-      </c>
-      <c r="L81" t="inlineStr"/>
+        <v>74</v>
+      </c>
+      <c r="L81" t="n">
+        <v>1.25</v>
+      </c>
       <c r="M81" t="n">
         <v>74.84</v>
       </c>
       <c r="N81" t="n">
-        <v>78.90000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
@@ -5286,30 +5242,30 @@
         <v>4</v>
       </c>
       <c r="G82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Alpha Capture (IRE)</t>
+          <t>Aberama Gold</t>
         </is>
       </c>
       <c r="I82" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J82" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="K82" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="L82" t="n">
-        <v>1.25</v>
+        <v>5.25</v>
       </c>
       <c r="M82" t="n">
         <v>74.84</v>
       </c>
       <c r="N82" t="n">
-        <v>78.09999999999999</v>
+        <v>69.3</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
@@ -5346,30 +5302,30 @@
         <v>4</v>
       </c>
       <c r="G83" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Aberama Gold</t>
+          <t>The Good Biscuit</t>
         </is>
       </c>
       <c r="I83" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J83" t="n">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="K83" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L83" t="n">
-        <v>5.25</v>
+        <v>5.75</v>
       </c>
       <c r="M83" t="n">
         <v>74.84</v>
       </c>
       <c r="N83" t="n">
-        <v>69.3</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -5406,30 +5362,30 @@
         <v>4</v>
       </c>
       <c r="G84" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>The Good Biscuit</t>
+          <t>Emperor Caradoc (FR)</t>
         </is>
       </c>
       <c r="I84" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J84" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K84" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L84" t="n">
-        <v>5.75</v>
+        <v>7.25</v>
       </c>
       <c r="M84" t="n">
         <v>74.84</v>
       </c>
       <c r="N84" t="n">
-        <v>67.09999999999999</v>
+        <v>61.3</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
@@ -5466,30 +5422,30 @@
         <v>4</v>
       </c>
       <c r="G85" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Emperor Caradoc (FR)</t>
+          <t>Maris Angel</t>
         </is>
       </c>
       <c r="I85" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J85" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K85" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L85" t="n">
-        <v>7.25</v>
+        <v>8</v>
       </c>
       <c r="M85" t="n">
         <v>74.84</v>
       </c>
       <c r="N85" t="n">
-        <v>61.3</v>
+        <v>60.6</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
@@ -5526,30 +5482,30 @@
         <v>4</v>
       </c>
       <c r="G86" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Maris Angel</t>
+          <t>Mr Cool (IRE)</t>
         </is>
       </c>
       <c r="I86" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J86" t="n">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="K86" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="L86" t="n">
-        <v>8</v>
+        <v>8.15</v>
       </c>
       <c r="M86" t="n">
         <v>74.84</v>
       </c>
       <c r="N86" t="n">
-        <v>60.6</v>
+        <v>48.8</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
@@ -5586,30 +5542,30 @@
         <v>4</v>
       </c>
       <c r="G87" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Mr Cool (IRE)</t>
+          <t>Dashing Dick (IRE)</t>
         </is>
       </c>
       <c r="I87" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J87" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="K87" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="L87" t="n">
-        <v>8.15</v>
+        <v>10.65</v>
       </c>
       <c r="M87" t="n">
         <v>74.84</v>
       </c>
       <c r="N87" t="n">
-        <v>50.4</v>
+        <v>42.7</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -5646,30 +5602,30 @@
         <v>4</v>
       </c>
       <c r="G88" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Dashing Dick (IRE)</t>
+          <t>Bravo Zulu (IRE)</t>
         </is>
       </c>
       <c r="I88" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J88" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K88" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L88" t="n">
-        <v>10.65</v>
+        <v>17.65</v>
       </c>
       <c r="M88" t="n">
         <v>74.84</v>
       </c>
       <c r="N88" t="n">
-        <v>47.6</v>
+        <v>29</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -5705,40 +5661,24 @@
       <c r="F89" t="n">
         <v>4</v>
       </c>
-      <c r="G89" t="n">
-        <v>9</v>
-      </c>
+      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Bravo Zulu (IRE)</t>
-        </is>
-      </c>
-      <c r="I89" t="n">
-        <v>5</v>
-      </c>
-      <c r="J89" t="n">
-        <v>132</v>
-      </c>
-      <c r="K89" t="n">
-        <v>76</v>
-      </c>
-      <c r="L89" t="n">
-        <v>17.65</v>
-      </c>
-      <c r="M89" t="n">
-        <v>74.84</v>
-      </c>
-      <c r="N89" t="n">
-        <v>29</v>
-      </c>
+          <t>Irish Nectar</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P89" t="n">
-        <v>0</v>
-      </c>
+      <c r="P89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5895,7 +5835,7 @@
         <v>4</v>
       </c>
       <c r="J92" t="n">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="K92" t="n">
         <v>74</v>
@@ -5907,7 +5847,7 @@
         <v>75.53</v>
       </c>
       <c r="N92" t="n">
-        <v>76.90000000000001</v>
+        <v>74.3</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -6553,7 +6493,7 @@
         <v>8</v>
       </c>
       <c r="J103" t="n">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="K103" t="n">
         <v>62</v>
@@ -6565,7 +6505,7 @@
         <v>133.52</v>
       </c>
       <c r="N103" t="n">
-        <v>55.2</v>
+        <v>47.9</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -6573,7 +6513,7 @@
         </is>
       </c>
       <c r="P103" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="104">
@@ -6633,7 +6573,7 @@
         </is>
       </c>
       <c r="P104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -6851,7 +6791,7 @@
         <v>3</v>
       </c>
       <c r="J108" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="K108" t="n">
         <v>72</v>
@@ -6863,7 +6803,7 @@
         <v>61.76</v>
       </c>
       <c r="N108" t="n">
-        <v>81.2</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -6911,7 +6851,7 @@
         <v>3</v>
       </c>
       <c r="J109" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="K109" t="n">
         <v>72</v>
@@ -6923,7 +6863,7 @@
         <v>61.76</v>
       </c>
       <c r="N109" t="n">
-        <v>73.8</v>
+        <v>69.3</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -6971,7 +6911,7 @@
         <v>3</v>
       </c>
       <c r="J110" t="n">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="K110" t="n">
         <v>69</v>
@@ -6983,7 +6923,7 @@
         <v>61.76</v>
       </c>
       <c r="N110" t="n">
-        <v>61.8</v>
+        <v>56.6</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7867,7 +7807,7 @@
         <v>5</v>
       </c>
       <c r="J125" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="K125" t="n">
         <v>48</v>
@@ -7879,7 +7819,7 @@
         <v>88.3</v>
       </c>
       <c r="N125" t="n">
-        <v>46.5</v>
+        <v>43</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -7927,7 +7867,7 @@
         <v>3</v>
       </c>
       <c r="J126" t="n">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="K126" t="n">
         <v>44</v>
@@ -7939,7 +7879,7 @@
         <v>88.3</v>
       </c>
       <c r="N126" t="n">
-        <v>41.7</v>
+        <v>36.8</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7947,7 +7887,7 @@
         </is>
       </c>
       <c r="P126" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="127">
@@ -8007,7 +7947,7 @@
         </is>
       </c>
       <c r="P127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128">
@@ -8107,7 +8047,7 @@
         <v>5</v>
       </c>
       <c r="J129" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="K129" t="n">
         <v>46</v>
@@ -8119,7 +8059,7 @@
         <v>88.3</v>
       </c>
       <c r="N129" t="n">
-        <v>28.8</v>
+        <v>25.6</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8167,7 +8107,7 @@
         <v>5</v>
       </c>
       <c r="J130" t="n">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K130" t="n">
         <v>48</v>
@@ -8179,7 +8119,7 @@
         <v>88.3</v>
       </c>
       <c r="N130" t="n">
-        <v>16.4</v>
+        <v>13.7</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -8651,7 +8591,7 @@
         <v>44</v>
       </c>
       <c r="L138" t="n">
-        <v>4.7</v>
+        <v>4.699999999999999</v>
       </c>
       <c r="M138" t="n">
         <v>88.34999999999999</v>
@@ -8711,7 +8651,7 @@
         <v>45</v>
       </c>
       <c r="L139" t="n">
-        <v>5.7</v>
+        <v>5.699999999999999</v>
       </c>
       <c r="M139" t="n">
         <v>88.34999999999999</v>
@@ -8765,7 +8705,7 @@
         <v>6</v>
       </c>
       <c r="J140" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="K140" t="n">
         <v>46</v>
@@ -8777,7 +8717,7 @@
         <v>88.34999999999999</v>
       </c>
       <c r="N140" t="n">
-        <v>-12.5</v>
+        <v>-14.9</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9412,18 +9352,18 @@
         <v>6</v>
       </c>
       <c r="G151" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>Sorted (IRE)</t>
+          <t>Lady Of Clover (IRE)</t>
         </is>
       </c>
       <c r="I151" t="n">
         <v>3</v>
       </c>
       <c r="J151" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="K151" t="n">
         <v>49</v>
@@ -9432,14 +9372,16 @@
       <c r="M151" t="n">
         <v>112.84</v>
       </c>
-      <c r="N151" t="inlineStr"/>
+      <c r="N151" t="n">
+        <v>20.3</v>
+      </c>
       <c r="O151" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P151" t="n">
-        <v>-13</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="152">
@@ -9468,28 +9410,30 @@
         <v>6</v>
       </c>
       <c r="G152" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>Lady Of Clover (IRE)</t>
+          <t>Knightmare (IRE)</t>
         </is>
       </c>
       <c r="I152" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J152" t="n">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="K152" t="n">
-        <v>49</v>
-      </c>
-      <c r="L152" t="inlineStr"/>
+        <v>50</v>
+      </c>
+      <c r="L152" t="n">
+        <v>1.25</v>
+      </c>
       <c r="M152" t="n">
         <v>112.84</v>
       </c>
       <c r="N152" t="n">
-        <v>23.3</v>
+        <v>22.8</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -9497,7 +9441,7 @@
         </is>
       </c>
       <c r="P152" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="153">
@@ -9526,15 +9470,15 @@
         <v>6</v>
       </c>
       <c r="G153" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>Knightmare (IRE)</t>
+          <t>Ciotog (IRE)</t>
         </is>
       </c>
       <c r="I153" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J153" t="n">
         <v>135</v>
@@ -9543,13 +9487,13 @@
         <v>50</v>
       </c>
       <c r="L153" t="n">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="M153" t="n">
         <v>112.84</v>
       </c>
       <c r="N153" t="n">
-        <v>22.8</v>
+        <v>20.7</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -9586,30 +9530,30 @@
         <v>6</v>
       </c>
       <c r="G154" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>Ciotog (IRE)</t>
+          <t>Rogers Dream</t>
         </is>
       </c>
       <c r="I154" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J154" t="n">
         <v>135</v>
       </c>
       <c r="K154" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="L154" t="n">
-        <v>2.5</v>
+        <v>2.65</v>
       </c>
       <c r="M154" t="n">
         <v>112.84</v>
       </c>
       <c r="N154" t="n">
-        <v>20.7</v>
+        <v>21</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -9617,7 +9561,7 @@
         </is>
       </c>
       <c r="P154" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="155">
@@ -9646,30 +9590,30 @@
         <v>6</v>
       </c>
       <c r="G155" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Rogers Dream</t>
+          <t>Lady Delila (IRE)</t>
         </is>
       </c>
       <c r="I155" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J155" t="n">
         <v>135</v>
       </c>
       <c r="K155" t="n">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="L155" t="n">
-        <v>2.65</v>
+        <v>3.4</v>
       </c>
       <c r="M155" t="n">
         <v>112.84</v>
       </c>
       <c r="N155" t="n">
-        <v>21</v>
+        <v>19.3</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -9677,7 +9621,7 @@
         </is>
       </c>
       <c r="P155" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156">
@@ -9706,30 +9650,30 @@
         <v>6</v>
       </c>
       <c r="G156" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Lady Delila (IRE)</t>
+          <t>Pams Sonnet</t>
         </is>
       </c>
       <c r="I156" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J156" t="n">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="K156" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L156" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="M156" t="n">
         <v>112.84</v>
       </c>
       <c r="N156" t="n">
-        <v>19.3</v>
+        <v>15.1</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -9766,11 +9710,11 @@
         <v>6</v>
       </c>
       <c r="G157" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Pams Sonnet</t>
+          <t>Thomas Tallis</t>
         </is>
       </c>
       <c r="I157" t="n">
@@ -9780,16 +9724,16 @@
         <v>123</v>
       </c>
       <c r="K157" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="L157" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="M157" t="n">
         <v>112.84</v>
       </c>
       <c r="N157" t="n">
-        <v>15.1</v>
+        <v>13.7</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -9826,30 +9770,30 @@
         <v>6</v>
       </c>
       <c r="G158" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Thomas Tallis</t>
+          <t>Lady Aiyana</t>
         </is>
       </c>
       <c r="I158" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J158" t="n">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="K158" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="L158" t="n">
-        <v>4</v>
+        <v>5.25</v>
       </c>
       <c r="M158" t="n">
         <v>112.84</v>
       </c>
       <c r="N158" t="n">
-        <v>13.7</v>
+        <v>13.5</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -9886,30 +9830,30 @@
         <v>6</v>
       </c>
       <c r="G159" t="n">
+        <v>9</v>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Raise The Stakes (IRE)</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>3</v>
+      </c>
+      <c r="J159" t="n">
+        <v>123</v>
+      </c>
+      <c r="K159" t="n">
+        <v>50</v>
+      </c>
+      <c r="L159" t="n">
         <v>8</v>
-      </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>Lady Aiyana</t>
-        </is>
-      </c>
-      <c r="I159" t="n">
-        <v>4</v>
-      </c>
-      <c r="J159" t="n">
-        <v>135</v>
-      </c>
-      <c r="K159" t="n">
-        <v>48</v>
-      </c>
-      <c r="L159" t="n">
-        <v>5.25</v>
       </c>
       <c r="M159" t="n">
         <v>112.84</v>
       </c>
       <c r="N159" t="n">
-        <v>13.5</v>
+        <v>-0.9</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -9946,11 +9890,11 @@
         <v>6</v>
       </c>
       <c r="G160" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Raise The Stakes (IRE)</t>
+          <t>Northern Soldier (IRE)</t>
         </is>
       </c>
       <c r="I160" t="n">
@@ -9960,16 +9904,16 @@
         <v>123</v>
       </c>
       <c r="K160" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="L160" t="n">
-        <v>8</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="M160" t="n">
         <v>112.84</v>
       </c>
       <c r="N160" t="n">
-        <v>-0.9</v>
+        <v>-1.8</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10006,11 +9950,11 @@
         <v>6</v>
       </c>
       <c r="G161" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Northern Soldier (IRE)</t>
+          <t>A Daughters Love</t>
         </is>
       </c>
       <c r="I161" t="n">
@@ -10020,16 +9964,16 @@
         <v>123</v>
       </c>
       <c r="K161" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="L161" t="n">
-        <v>8.050000000000001</v>
+        <v>11.3</v>
       </c>
       <c r="M161" t="n">
         <v>112.84</v>
       </c>
       <c r="N161" t="n">
-        <v>-1.8</v>
+        <v>-12.6</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10066,11 +10010,11 @@
         <v>6</v>
       </c>
       <c r="G162" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>A Daughters Love</t>
+          <t>Antique Blue (IRE)</t>
         </is>
       </c>
       <c r="I162" t="n">
@@ -10080,16 +10024,16 @@
         <v>123</v>
       </c>
       <c r="K162" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="L162" t="n">
-        <v>11.3</v>
+        <v>12.3</v>
       </c>
       <c r="M162" t="n">
         <v>112.84</v>
       </c>
       <c r="N162" t="n">
-        <v>-12.6</v>
+        <v>-15.4</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -10125,40 +10069,24 @@
       <c r="F163" t="n">
         <v>6</v>
       </c>
-      <c r="G163" t="n">
-        <v>12</v>
-      </c>
+      <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Antique Blue (IRE)</t>
-        </is>
-      </c>
-      <c r="I163" t="n">
-        <v>3</v>
-      </c>
-      <c r="J163" t="n">
-        <v>123</v>
-      </c>
-      <c r="K163" t="n">
-        <v>46</v>
-      </c>
-      <c r="L163" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="M163" t="n">
-        <v>112.84</v>
-      </c>
-      <c r="N163" t="n">
-        <v>-15.4</v>
-      </c>
+          <t>Sorted (IRE)</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr"/>
+      <c r="L163" t="inlineStr"/>
+      <c r="M163" t="inlineStr"/>
+      <c r="N163" t="inlineStr"/>
       <c r="O163" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P163" t="n">
-        <v>0</v>
-      </c>
+      <c r="P163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -10186,34 +10114,36 @@
         <v>6</v>
       </c>
       <c r="G164" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Thehunnebelllegacy</t>
+          <t>South Coast Star (IRE)</t>
         </is>
       </c>
       <c r="I164" t="n">
         <v>3</v>
       </c>
       <c r="J164" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K164" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="n">
         <v>87.98999999999999</v>
       </c>
-      <c r="N164" t="inlineStr"/>
+      <c r="N164" t="n">
+        <v>68.7</v>
+      </c>
       <c r="O164" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P164" t="n">
-        <v>-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165">
@@ -10242,28 +10172,30 @@
         <v>6</v>
       </c>
       <c r="G165" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>South Coast Star (IRE)</t>
+          <t>Distillation (FR)</t>
         </is>
       </c>
       <c r="I165" t="n">
         <v>3</v>
       </c>
       <c r="J165" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K165" t="n">
-        <v>53</v>
-      </c>
-      <c r="L165" t="inlineStr"/>
+        <v>52</v>
+      </c>
+      <c r="L165" t="n">
+        <v>6</v>
+      </c>
       <c r="M165" t="n">
         <v>87.98999999999999</v>
       </c>
       <c r="N165" t="n">
-        <v>68.7</v>
+        <v>50.5</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -10271,7 +10203,7 @@
         </is>
       </c>
       <c r="P165" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="166">
@@ -10300,30 +10232,30 @@
         <v>6</v>
       </c>
       <c r="G166" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Distillation (FR)</t>
+          <t>Stole My Heart (IRE)</t>
         </is>
       </c>
       <c r="I166" t="n">
         <v>3</v>
       </c>
       <c r="J166" t="n">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="K166" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="L166" t="n">
-        <v>6</v>
+        <v>7.25</v>
       </c>
       <c r="M166" t="n">
         <v>87.98999999999999</v>
       </c>
       <c r="N166" t="n">
-        <v>50.5</v>
+        <v>53.2</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -10331,7 +10263,7 @@
         </is>
       </c>
       <c r="P166" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
@@ -10360,11 +10292,11 @@
         <v>6</v>
       </c>
       <c r="G167" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Stole My Heart (IRE)</t>
+          <t>Amazing Anita</t>
         </is>
       </c>
       <c r="I167" t="n">
@@ -10377,13 +10309,13 @@
         <v>57</v>
       </c>
       <c r="L167" t="n">
-        <v>7.25</v>
+        <v>7.4</v>
       </c>
       <c r="M167" t="n">
         <v>87.98999999999999</v>
       </c>
       <c r="N167" t="n">
-        <v>53.2</v>
+        <v>52.2</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -10420,30 +10352,30 @@
         <v>6</v>
       </c>
       <c r="G168" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Amazing Anita</t>
+          <t>Lady Vanguard</t>
         </is>
       </c>
       <c r="I168" t="n">
         <v>3</v>
       </c>
       <c r="J168" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K168" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L168" t="n">
-        <v>7.4</v>
+        <v>10.65</v>
       </c>
       <c r="M168" t="n">
         <v>87.98999999999999</v>
       </c>
       <c r="N168" t="n">
-        <v>52.2</v>
+        <v>42.4</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -10451,7 +10383,7 @@
         </is>
       </c>
       <c r="P168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169">
@@ -10480,30 +10412,30 @@
         <v>6</v>
       </c>
       <c r="G169" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Lady Vanguard</t>
+          <t>Zoulette (IRE)</t>
         </is>
       </c>
       <c r="I169" t="n">
         <v>3</v>
       </c>
       <c r="J169" t="n">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="K169" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="L169" t="n">
-        <v>10.65</v>
+        <v>12.4</v>
       </c>
       <c r="M169" t="n">
         <v>87.98999999999999</v>
       </c>
       <c r="N169" t="n">
-        <v>42.4</v>
+        <v>36.4</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -10540,30 +10472,30 @@
         <v>6</v>
       </c>
       <c r="G170" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Zoulette (IRE)</t>
+          <t>Veld (IRE)</t>
         </is>
       </c>
       <c r="I170" t="n">
         <v>3</v>
       </c>
       <c r="J170" t="n">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="K170" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="L170" t="n">
-        <v>12.4</v>
+        <v>15.65</v>
       </c>
       <c r="M170" t="n">
         <v>87.98999999999999</v>
       </c>
       <c r="N170" t="n">
-        <v>36.4</v>
+        <v>31.3</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -10600,30 +10532,30 @@
         <v>6</v>
       </c>
       <c r="G171" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Veld (IRE)</t>
+          <t>City Of Dreams (IRE)</t>
         </is>
       </c>
       <c r="I171" t="n">
         <v>3</v>
       </c>
       <c r="J171" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="K171" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="L171" t="n">
-        <v>15.65</v>
+        <v>16.65</v>
       </c>
       <c r="M171" t="n">
         <v>87.98999999999999</v>
       </c>
       <c r="N171" t="n">
-        <v>31.3</v>
+        <v>25.1</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -10660,34 +10592,34 @@
         <v>6</v>
       </c>
       <c r="G172" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>City Of Dreams (IRE)</t>
+          <t>Enduring Story</t>
         </is>
       </c>
       <c r="I172" t="n">
         <v>3</v>
       </c>
       <c r="J172" t="n">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="K172" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="L172" t="n">
-        <v>16.65</v>
+        <v>32.65</v>
       </c>
       <c r="M172" t="n">
         <v>87.98999999999999</v>
       </c>
       <c r="N172" t="n">
-        <v>25.1</v>
+        <v>-14.2</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="P172" t="n">
@@ -10719,40 +10651,24 @@
       <c r="F173" t="n">
         <v>6</v>
       </c>
-      <c r="G173" t="n">
-        <v>9</v>
-      </c>
+      <c r="G173" t="inlineStr"/>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Enduring Story</t>
-        </is>
-      </c>
-      <c r="I173" t="n">
-        <v>3</v>
-      </c>
-      <c r="J173" t="n">
-        <v>121</v>
-      </c>
-      <c r="K173" t="n">
-        <v>45</v>
-      </c>
-      <c r="L173" t="n">
-        <v>32.65</v>
-      </c>
-      <c r="M173" t="n">
-        <v>87.98999999999999</v>
-      </c>
-      <c r="N173" t="n">
-        <v>-14.2</v>
-      </c>
+          <t>Thehunnebelllegacy</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="inlineStr"/>
+      <c r="N173" t="inlineStr"/>
       <c r="O173" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="P173" t="n">
-        <v>0</v>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -10780,34 +10696,36 @@
         <v>6</v>
       </c>
       <c r="G174" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Ndoto</t>
+          <t>Based (IRE)</t>
         </is>
       </c>
       <c r="I174" t="n">
         <v>3</v>
       </c>
       <c r="J174" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K174" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="L174" t="inlineStr"/>
       <c r="M174" t="n">
         <v>89.04000000000001</v>
       </c>
-      <c r="N174" t="inlineStr"/>
+      <c r="N174" t="n">
+        <v>58</v>
+      </c>
       <c r="O174" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P174" t="n">
-        <v>-9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175">
@@ -10836,28 +10754,30 @@
         <v>6</v>
       </c>
       <c r="G175" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>Based (IRE)</t>
+          <t>Musical Soldier (IRE)</t>
         </is>
       </c>
       <c r="I175" t="n">
         <v>3</v>
       </c>
       <c r="J175" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K175" t="n">
-        <v>53</v>
-      </c>
-      <c r="L175" t="inlineStr"/>
+        <v>55</v>
+      </c>
+      <c r="L175" t="n">
+        <v>2</v>
+      </c>
       <c r="M175" t="n">
         <v>89.04000000000001</v>
       </c>
       <c r="N175" t="n">
-        <v>58</v>
+        <v>55.4</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -10894,30 +10814,30 @@
         <v>6</v>
       </c>
       <c r="G176" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Musical Soldier (IRE)</t>
+          <t>Labiche</t>
         </is>
       </c>
       <c r="I176" t="n">
         <v>3</v>
       </c>
       <c r="J176" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K176" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L176" t="n">
-        <v>2</v>
+        <v>3.75</v>
       </c>
       <c r="M176" t="n">
         <v>89.04000000000001</v>
       </c>
       <c r="N176" t="n">
-        <v>55.4</v>
+        <v>49.3</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -10954,30 +10874,30 @@
         <v>6</v>
       </c>
       <c r="G177" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Labiche</t>
+          <t>Electrocution</t>
         </is>
       </c>
       <c r="I177" t="n">
         <v>3</v>
       </c>
       <c r="J177" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K177" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L177" t="n">
-        <v>3.75</v>
+        <v>4.5</v>
       </c>
       <c r="M177" t="n">
         <v>89.04000000000001</v>
       </c>
       <c r="N177" t="n">
-        <v>49.3</v>
+        <v>45.9</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -10985,7 +10905,7 @@
         </is>
       </c>
       <c r="P177" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="178">
@@ -11014,30 +10934,30 @@
         <v>6</v>
       </c>
       <c r="G178" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Electrocution</t>
+          <t>Dusk Damsel</t>
         </is>
       </c>
       <c r="I178" t="n">
         <v>3</v>
       </c>
       <c r="J178" t="n">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="K178" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="L178" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="M178" t="n">
         <v>89.04000000000001</v>
       </c>
       <c r="N178" t="n">
-        <v>45.9</v>
+        <v>47.3</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -11045,7 +10965,7 @@
         </is>
       </c>
       <c r="P178" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="179">
@@ -11074,30 +10994,30 @@
         <v>6</v>
       </c>
       <c r="G179" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Dusk Damsel</t>
+          <t>Power Of Chora (IRE)</t>
         </is>
       </c>
       <c r="I179" t="n">
         <v>3</v>
       </c>
       <c r="J179" t="n">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="K179" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L179" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="M179" t="n">
         <v>89.04000000000001</v>
       </c>
       <c r="N179" t="n">
-        <v>47.3</v>
+        <v>36.7</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -11105,7 +11025,7 @@
         </is>
       </c>
       <c r="P179" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="180">
@@ -11134,30 +11054,30 @@
         <v>6</v>
       </c>
       <c r="G180" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Power Of Chora (IRE)</t>
+          <t>Inclusive</t>
         </is>
       </c>
       <c r="I180" t="n">
         <v>3</v>
       </c>
       <c r="J180" t="n">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="K180" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L180" t="n">
-        <v>6.5</v>
+        <v>8.25</v>
       </c>
       <c r="M180" t="n">
         <v>89.04000000000001</v>
       </c>
       <c r="N180" t="n">
-        <v>42.8</v>
+        <v>32.5</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -11165,7 +11085,7 @@
         </is>
       </c>
       <c r="P180" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="181">
@@ -11194,30 +11114,30 @@
         <v>6</v>
       </c>
       <c r="G181" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Inclusive</t>
+          <t>Warriors Choice</t>
         </is>
       </c>
       <c r="I181" t="n">
         <v>3</v>
       </c>
       <c r="J181" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="K181" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L181" t="n">
-        <v>8.25</v>
+        <v>9</v>
       </c>
       <c r="M181" t="n">
         <v>89.04000000000001</v>
       </c>
       <c r="N181" t="n">
-        <v>37.4</v>
+        <v>36.8</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -11225,7 +11145,7 @@
         </is>
       </c>
       <c r="P181" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="182">
@@ -11253,40 +11173,24 @@
       <c r="F182" t="n">
         <v>6</v>
       </c>
-      <c r="G182" t="n">
-        <v>8</v>
-      </c>
+      <c r="G182" t="inlineStr"/>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Warriors Choice</t>
-        </is>
-      </c>
-      <c r="I182" t="n">
-        <v>3</v>
-      </c>
-      <c r="J182" t="n">
-        <v>133</v>
-      </c>
-      <c r="K182" t="n">
-        <v>57</v>
-      </c>
-      <c r="L182" t="n">
-        <v>9</v>
-      </c>
-      <c r="M182" t="n">
-        <v>89.04000000000001</v>
-      </c>
-      <c r="N182" t="n">
-        <v>36.8</v>
-      </c>
+          <t>Ndoto</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr"/>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr"/>
+      <c r="M182" t="inlineStr"/>
+      <c r="N182" t="inlineStr"/>
       <c r="O182" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P182" t="n">
-        <v>0</v>
-      </c>
+      <c r="P182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -11314,34 +11218,36 @@
         <v>6</v>
       </c>
       <c r="G183" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>Age Of Time (FR)</t>
+          <t>Beachborough Girl</t>
         </is>
       </c>
       <c r="I183" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J183" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K183" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="L183" t="inlineStr"/>
       <c r="M183" t="n">
         <v>120.51</v>
       </c>
-      <c r="N183" t="inlineStr"/>
+      <c r="N183" t="n">
+        <v>55.7</v>
+      </c>
       <c r="O183" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P183" t="n">
-        <v>-12</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="184">
@@ -11370,28 +11276,30 @@
         <v>6</v>
       </c>
       <c r="G184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Beachborough Girl</t>
+          <t>Study Up</t>
         </is>
       </c>
       <c r="I184" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J184" t="n">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="K184" t="n">
-        <v>60</v>
-      </c>
-      <c r="L184" t="inlineStr"/>
+        <v>65</v>
+      </c>
+      <c r="L184" t="n">
+        <v>0.05</v>
+      </c>
       <c r="M184" t="n">
         <v>120.51</v>
       </c>
       <c r="N184" t="n">
-        <v>55.7</v>
+        <v>59.5</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -11399,7 +11307,7 @@
         </is>
       </c>
       <c r="P184" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185">
@@ -11428,30 +11336,30 @@
         <v>6</v>
       </c>
       <c r="G185" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>Study Up</t>
+          <t>Roman Secret (IRE)</t>
         </is>
       </c>
       <c r="I185" t="n">
         <v>5</v>
       </c>
       <c r="J185" t="n">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="K185" t="n">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="L185" t="n">
-        <v>0.05</v>
+        <v>1.55</v>
       </c>
       <c r="M185" t="n">
         <v>120.51</v>
       </c>
       <c r="N185" t="n">
-        <v>59.5</v>
+        <v>48.5</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -11459,7 +11367,7 @@
         </is>
       </c>
       <c r="P185" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="186">
@@ -11488,30 +11396,30 @@
         <v>6</v>
       </c>
       <c r="G186" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>Roman Secret (IRE)</t>
+          <t>Poke The Bear (IRE)</t>
         </is>
       </c>
       <c r="I186" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J186" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K186" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L186" t="n">
-        <v>1.55</v>
+        <v>1.7</v>
       </c>
       <c r="M186" t="n">
         <v>120.51</v>
       </c>
       <c r="N186" t="n">
-        <v>48.5</v>
+        <v>50.4</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -11519,7 +11427,7 @@
         </is>
       </c>
       <c r="P186" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="187">
@@ -11548,30 +11456,30 @@
         <v>6</v>
       </c>
       <c r="G187" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Poke The Bear (IRE)</t>
+          <t>Silkies Sib (IRE)</t>
         </is>
       </c>
       <c r="I187" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J187" t="n">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K187" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L187" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="M187" t="n">
         <v>120.51</v>
       </c>
       <c r="N187" t="n">
-        <v>50.4</v>
+        <v>47</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -11579,7 +11487,7 @@
         </is>
       </c>
       <c r="P187" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="188">
@@ -11608,30 +11516,30 @@
         <v>6</v>
       </c>
       <c r="G188" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>Silkies Sib (IRE)</t>
+          <t>City Escape (IRE)</t>
         </is>
       </c>
       <c r="I188" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J188" t="n">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K188" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L188" t="n">
-        <v>2.2</v>
+        <v>2.25</v>
       </c>
       <c r="M188" t="n">
         <v>120.51</v>
       </c>
       <c r="N188" t="n">
-        <v>47</v>
+        <v>44.5</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -11668,30 +11576,30 @@
         <v>6</v>
       </c>
       <c r="G189" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>City Escape (IRE)</t>
+          <t>Arlecchinos Rex</t>
         </is>
       </c>
       <c r="I189" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J189" t="n">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K189" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="L189" t="n">
-        <v>2.25</v>
+        <v>3.5</v>
       </c>
       <c r="M189" t="n">
         <v>120.51</v>
       </c>
       <c r="N189" t="n">
-        <v>44.5</v>
+        <v>39.6</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -11728,30 +11636,30 @@
         <v>6</v>
       </c>
       <c r="G190" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>Arlecchinos Rex</t>
+          <t>Port Noir</t>
         </is>
       </c>
       <c r="I190" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J190" t="n">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K190" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="L190" t="n">
-        <v>3.5</v>
+        <v>4.75</v>
       </c>
       <c r="M190" t="n">
         <v>120.51</v>
       </c>
       <c r="N190" t="n">
-        <v>39.6</v>
+        <v>32</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -11759,7 +11667,7 @@
         </is>
       </c>
       <c r="P190" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="191">
@@ -11788,30 +11696,30 @@
         <v>6</v>
       </c>
       <c r="G191" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>Port Noir</t>
+          <t>Luan (FR)</t>
         </is>
       </c>
       <c r="I191" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J191" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K191" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L191" t="n">
-        <v>4.75</v>
+        <v>5.75</v>
       </c>
       <c r="M191" t="n">
         <v>120.51</v>
       </c>
       <c r="N191" t="n">
-        <v>39.4</v>
+        <v>32.5</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -11819,7 +11727,7 @@
         </is>
       </c>
       <c r="P191" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192">
@@ -11848,30 +11756,30 @@
         <v>6</v>
       </c>
       <c r="G192" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>Luan (FR)</t>
+          <t>Cherry Hill</t>
         </is>
       </c>
       <c r="I192" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J192" t="n">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="K192" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="L192" t="n">
-        <v>5.75</v>
+        <v>9.25</v>
       </c>
       <c r="M192" t="n">
         <v>120.51</v>
       </c>
       <c r="N192" t="n">
-        <v>32.5</v>
+        <v>23</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -11908,30 +11816,30 @@
         <v>6</v>
       </c>
       <c r="G193" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>Cherry Hill</t>
+          <t>Shaws Phoenix (IRE)</t>
         </is>
       </c>
       <c r="I193" t="n">
         <v>5</v>
       </c>
       <c r="J193" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K193" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="L193" t="n">
-        <v>9.25</v>
+        <v>15.75</v>
       </c>
       <c r="M193" t="n">
         <v>120.51</v>
       </c>
       <c r="N193" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -11967,40 +11875,24 @@
       <c r="F194" t="n">
         <v>6</v>
       </c>
-      <c r="G194" t="n">
-        <v>11</v>
-      </c>
+      <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr">
         <is>
-          <t>Shaws Phoenix (IRE)</t>
-        </is>
-      </c>
-      <c r="I194" t="n">
-        <v>5</v>
-      </c>
-      <c r="J194" t="n">
-        <v>125</v>
-      </c>
-      <c r="K194" t="n">
-        <v>50</v>
-      </c>
-      <c r="L194" t="n">
-        <v>15.75</v>
-      </c>
-      <c r="M194" t="n">
-        <v>120.51</v>
-      </c>
-      <c r="N194" t="n">
-        <v>4.8</v>
-      </c>
+          <t>Age Of Time (FR)</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
+      <c r="L194" t="inlineStr"/>
+      <c r="M194" t="inlineStr"/>
+      <c r="N194" t="inlineStr"/>
       <c r="O194" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P194" t="n">
-        <v>0</v>
-      </c>
+      <c r="P194" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>